<commit_message>
Removed unwanted text in column I
</commit_message>
<xml_diff>
--- a/PMars_Testcases_Task1.xlsx
+++ b/PMars_Testcases_Task1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Eve Ombos\ProjectMars\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5571AB01-AD5B-412A-9B19-32D86255D299}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA660302-D14F-4855-877D-4E43A3A87091}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="14380" windowHeight="5180" xr2:uid="{C0D87ADB-D452-402E-8108-E51A4F556DCD}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="123">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -2870,9 +2870,6 @@
 * No limit was encountered during testing.
 </t>
     </r>
-  </si>
-  <si>
-    <t>Destructive Testing (Unexpected Use or Breaking Boundaries)</t>
   </si>
   <si>
     <t>Multiple Add Button Clicks</t>
@@ -3256,7 +3253,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45142E27-1A1D-464C-BB39-DEA7A0C7A942}">
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr defaultColWidth="23" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="22.08984375" style="2" bestFit="1" customWidth="1"/>
@@ -3269,7 +3266,7 @@
     <col min="8" max="16384" width="23" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3292,7 +3289,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
@@ -3315,7 +3312,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -3338,7 +3335,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
@@ -3361,7 +3358,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
@@ -3384,7 +3381,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>13</v>
       </c>
@@ -3407,7 +3404,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="188.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>14</v>
       </c>
@@ -3430,7 +3427,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>15</v>
       </c>
@@ -3452,11 +3449,8 @@
       <c r="G8" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="I8" s="2" t="s">
-        <v>119</v>
-      </c>
     </row>
-    <row r="9" spans="1:9" ht="304.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" ht="304.5" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>16</v>
       </c>
@@ -3479,7 +3473,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="116" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" ht="116" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>18</v>
       </c>
@@ -3502,30 +3496,30 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="270" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" ht="270" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>61</v>
       </c>
       <c r="D11" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="F11" s="2" t="s">
         <v>122</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>123</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>17</v>
       </c>
@@ -3548,7 +3542,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>60</v>
       </c>
@@ -3571,7 +3565,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="275.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>67</v>
       </c>
@@ -3594,7 +3588,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="174" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" ht="174" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>73</v>
       </c>
@@ -3617,7 +3611,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="188.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>77</v>
       </c>
@@ -3640,7 +3634,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>81</v>
       </c>
@@ -3663,7 +3657,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>94</v>
       </c>
@@ -3686,7 +3680,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>95</v>
       </c>
@@ -3709,7 +3703,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="203" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" ht="203" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>113</v>
       </c>
@@ -3732,7 +3726,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="145" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" ht="145" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
         <v>101</v>
       </c>
@@ -3754,11 +3748,8 @@
       <c r="G21" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="I21" s="2" t="s">
-        <v>119</v>
-      </c>
     </row>
-    <row r="22" spans="1:9" ht="217.5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>102</v>
       </c>

</xml_diff>

<commit_message>
Revert "Removed unwanted text in column I"
This reverts commit 7899ab29750fccd51cda81c35b5fec6c6fd49d6b.
</commit_message>
<xml_diff>
--- a/PMars_Testcases_Task1.xlsx
+++ b/PMars_Testcases_Task1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Eve Ombos\ProjectMars\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA660302-D14F-4855-877D-4E43A3A87091}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5571AB01-AD5B-412A-9B19-32D86255D299}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="14380" windowHeight="5180" xr2:uid="{C0D87ADB-D452-402E-8108-E51A4F556DCD}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="124">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -2870,6 +2870,9 @@
 * No limit was encountered during testing.
 </t>
     </r>
+  </si>
+  <si>
+    <t>Destructive Testing (Unexpected Use or Breaking Boundaries)</t>
   </si>
   <si>
     <t>Multiple Add Button Clicks</t>
@@ -3253,7 +3256,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45142E27-1A1D-464C-BB39-DEA7A0C7A942}">
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr defaultColWidth="23" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="22.08984375" style="2" bestFit="1" customWidth="1"/>
@@ -3266,7 +3269,7 @@
     <col min="8" max="16384" width="23" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3289,7 +3292,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
@@ -3312,7 +3315,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -3335,7 +3338,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
@@ -3358,7 +3361,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
@@ -3381,7 +3384,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>13</v>
       </c>
@@ -3404,7 +3407,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="188.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>14</v>
       </c>
@@ -3427,7 +3430,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>15</v>
       </c>
@@ -3449,8 +3452,11 @@
       <c r="G8" s="2" t="s">
         <v>8</v>
       </c>
+      <c r="I8" s="2" t="s">
+        <v>119</v>
+      </c>
     </row>
-    <row r="9" spans="1:7" ht="304.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" ht="304.5" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>16</v>
       </c>
@@ -3473,7 +3479,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="116" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" ht="116" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>18</v>
       </c>
@@ -3496,30 +3502,30 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="270" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" ht="270" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>61</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>17</v>
       </c>
@@ -3542,7 +3548,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>60</v>
       </c>
@@ -3565,7 +3571,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="275.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>67</v>
       </c>
@@ -3588,7 +3594,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="174" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" ht="174" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>73</v>
       </c>
@@ -3611,7 +3617,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="188.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>77</v>
       </c>
@@ -3634,7 +3640,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:9" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>81</v>
       </c>
@@ -3657,7 +3663,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:9" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>94</v>
       </c>
@@ -3680,7 +3686,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:9" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>95</v>
       </c>
@@ -3703,7 +3709,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="203" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:9" ht="203" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>113</v>
       </c>
@@ -3726,7 +3732,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="145" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:9" ht="145" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
         <v>101</v>
       </c>
@@ -3748,8 +3754,11 @@
       <c r="G21" s="2" t="s">
         <v>8</v>
       </c>
+      <c r="I21" s="2" t="s">
+        <v>119</v>
+      </c>
     </row>
-    <row r="22" spans="1:7" ht="217.5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:9" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>102</v>
       </c>

</xml_diff>